<commit_message>
Ya arregle el modificar en pago y ademas cambie cosas, y arregle lo de excel y otras cosas y el chexbox en pago
</commit_message>
<xml_diff>
--- a/Pagos.xlsx
+++ b/Pagos.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
   <si>
     <t>Material</t>
   </si>
@@ -24,31 +24,31 @@
     <t>Cantidad</t>
   </si>
   <si>
-    <t>33</t>
+    <t>d</t>
   </si>
   <si>
-    <t>mancipe</t>
+    <t>f</t>
   </si>
   <si>
-    <t>1200</t>
+    <t>ff</t>
   </si>
   <si>
-    <t>5</t>
+    <t>fff</t>
   </si>
   <si>
-    <t>nlk</t>
+    <t>gdgddgdg</t>
   </si>
   <si>
-    <t>lk</t>
+    <t>dgdgdg</t>
   </si>
   <si>
-    <t>kljkl</t>
+    <t>dgdgdgdgdgdgdgdgd</t>
   </si>
   <si>
     <t>Servicio</t>
   </si>
   <si>
-    <t>kevin</t>
+    <t>ffffff</t>
   </si>
 </sst>
 </file>
@@ -147,7 +147,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -163,13 +163,24 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mejore el boton de agregar y modificar ahorrando codigo
</commit_message>
<xml_diff>
--- a/Pagos.xlsx
+++ b/Pagos.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Material</t>
   </si>
@@ -24,31 +24,55 @@
     <t>Cantidad</t>
   </si>
   <si>
+    <t>ValorTotal</t>
+  </si>
+  <si>
     <t>d</t>
   </si>
   <si>
-    <t>f</t>
-  </si>
-  <si>
-    <t>ff</t>
-  </si>
-  <si>
-    <t>fff</t>
-  </si>
-  <si>
-    <t>gdgddgdg</t>
-  </si>
-  <si>
-    <t>dgdgdg</t>
-  </si>
-  <si>
-    <t>dgdgdgdgdgdgdgdgd</t>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>gg</t>
+  </si>
+  <si>
+    <t>30.00</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>900.0</t>
+  </si>
+  <si>
+    <t>3f</t>
+  </si>
+  <si>
+    <t>0.003</t>
+  </si>
+  <si>
+    <t>0.09</t>
   </si>
   <si>
     <t>Servicio</t>
   </si>
   <si>
-    <t>ffffff</t>
+    <t>2</t>
+  </si>
+  <si>
+    <t>20.00</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>400.0</t>
   </si>
 </sst>
 </file>
@@ -93,7 +117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -106,38 +130,50 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -147,12 +183,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -160,27 +196,22 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Termine de mostrar el valor total y ademas quite la x en el agregar
</commit_message>
<xml_diff>
--- a/Pagos.xlsx
+++ b/Pagos.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>Material</t>
   </si>
@@ -51,19 +51,28 @@
     <t>900.0</t>
   </si>
   <si>
+    <t>fghj</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>23.0</t>
+  </si>
+  <si>
+    <t>9.0</t>
+  </si>
+  <si>
     <t>Servicio</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>20.00</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>400.0</t>
+    <t>44</t>
+  </si>
+  <si>
+    <t>132.0</t>
   </si>
 </sst>
 </file>
@@ -108,7 +117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -151,6 +160,34 @@
       </c>
       <c r="D3" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -165,7 +202,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -179,16 +216,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cree inventario y cree la interfaz
</commit_message>
<xml_diff>
--- a/Pagos.xlsx
+++ b/Pagos.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <t>Material</t>
   </si>
@@ -27,52 +27,25 @@
     <t>ValorTotal</t>
   </si>
   <si>
-    <t>d</t>
+    <t>deee</t>
   </si>
   <si>
-    <t>3</t>
+    <t>33</t>
+  </si>
+  <si>
+    <t>1089.0</t>
+  </si>
+  <si>
+    <t>Servicio</t>
+  </si>
+  <si>
+    <t>f</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>ggddg</t>
-  </si>
-  <si>
-    <t>30.00</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>900.0</t>
-  </si>
-  <si>
-    <t>fghj</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>23.0</t>
-  </si>
-  <si>
-    <t>9.0</t>
-  </si>
-  <si>
-    <t>Servicio</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>132.0</t>
+    <t>16.0</t>
   </si>
 </sst>
 </file>
@@ -117,7 +90,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -142,52 +115,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -202,7 +133,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -216,16 +147,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hice lo de inventario, falta buscador y arregle un bug y retoque cosas
</commit_message>
<xml_diff>
--- a/Pagos.xlsx
+++ b/Pagos.xlsx
@@ -7,45 +7,59 @@
   </bookViews>
   <sheets>
     <sheet name="Materiales" r:id="rId3" sheetId="1"/>
-    <sheet name="Servicios" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
   <si>
-    <t>Material</t>
+    <t>FechaIngreso</t>
   </si>
   <si>
-    <t>Valor</t>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>FechaCompra</t>
   </si>
   <si>
     <t>Cantidad</t>
   </si>
   <si>
+    <t>ValorUnitario</t>
+  </si>
+  <si>
     <t>ValorTotal</t>
   </si>
   <si>
-    <t>deee</t>
+    <t>2024-10-31</t>
   </si>
   <si>
-    <t>33</t>
+    <t>3</t>
   </si>
   <si>
-    <t>1089.0</t>
+    <t>9.0</t>
   </si>
   <si>
-    <t>Servicio</t>
+    <t>2024-10-31  Hora:  02:38</t>
   </si>
   <si>
-    <t>f</t>
+    <t>ddd</t>
   </si>
   <si>
-    <t>4</t>
+    <t>31-10-2024</t>
   </si>
   <si>
-    <t>16.0</t>
+    <t>333333</t>
+  </si>
+  <si>
+    <t>33333</t>
+  </si>
+  <si>
+    <t>1.1110989E10</t>
+  </si>
+  <si>
+    <t>2024-10-31  Hora:  02:39</t>
   </si>
 </sst>
 </file>
@@ -90,7 +104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -106,57 +120,71 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="F1" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
-        <v>9</v>
+      <c r="B3" t="s">
+        <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>10</v>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agregue para que sea mover con enter en los menu de agregar y la opcion de borrar con delete y suprimi
</commit_message>
<xml_diff>
--- a/Pagos.xlsx
+++ b/Pagos.xlsx
@@ -7,36 +7,68 @@
   </bookViews>
   <sheets>
     <sheet name="Materiales" r:id="rId3" sheetId="1"/>
-    <sheet name="Servicios" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
-  <si>
-    <t>Fecha ingreso</t>
-  </si>
-  <si>
-    <t>Material</t>
-  </si>
-  <si>
-    <t>Fecha Compra</t>
-  </si>
-  <si>
-    <t>Valor</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+  <si>
+    <t>FechaIngreso</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>FechaCompra</t>
   </si>
   <si>
     <t>Cantidad</t>
   </si>
   <si>
+    <t>ValorUnitario</t>
+  </si>
+  <si>
     <t>ValorTotal</t>
   </si>
   <si>
-    <t>Fecha Ingreso</t>
-  </si>
-  <si>
-    <t>Servicio</t>
+    <t>2024-10-31  Hora:  12:02</t>
+  </si>
+  <si>
+    <t>cemento</t>
+  </si>
+  <si>
+    <t>2024-10-31</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>400000.0</t>
+  </si>
+  <si>
+    <t>tornillos</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>5000</t>
+  </si>
+  <si>
+    <t>100000.0</t>
+  </si>
+  <si>
+    <t>2024-10-31  Hora:  12:20</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>9.0</t>
   </si>
 </sst>
 </file>
@@ -81,7 +113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -104,34 +136,64 @@
         <v>5</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
+    <row r="2">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>